<commit_message>
Atualiza Preset/Situação de Sicario e Coleção Tipo de O Turista
</commit_message>
<xml_diff>
--- a/Cine Família B10 Completo.xlsx
+++ b/Cine Família B10 Completo.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FF028EA-D5EF-BA4B-887A-D51F9B8E1F6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF969C5B-41E1-314F-95CD-14EE7ADB5D35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="35420" windowHeight="21100" tabRatio="500" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="35420" windowHeight="21100" tabRatio="500" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Clássicos" sheetId="1" r:id="rId1"/>
@@ -15686,7 +15686,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="000"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color theme="1"/>
@@ -15773,12 +15773,6 @@
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -15806,7 +15800,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -15920,12 +15914,8 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -15940,26 +15930,30 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="3" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="3"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="fill"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="3" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="3" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="21" fontId="13" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="21" fontId="12" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="3" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="3" applyAlignment="1">
       <alignment horizontal="fill"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="3" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hiperlink" xfId="2" builtinId="8"/>
@@ -29104,933 +29098,933 @@
   <dimension ref="A1:U79"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" style="60" customWidth="1"/>
-    <col min="2" max="2" width="12.5" style="57" customWidth="1"/>
-    <col min="3" max="3" width="7.6640625" style="55" customWidth="1"/>
-    <col min="4" max="4" width="27.33203125" style="55" customWidth="1"/>
-    <col min="5" max="5" width="22.5" style="55" customWidth="1"/>
-    <col min="6" max="6" width="7.1640625" style="58" customWidth="1"/>
-    <col min="7" max="7" width="9" style="58" customWidth="1"/>
-    <col min="8" max="8" width="7.33203125" style="58" customWidth="1"/>
-    <col min="9" max="9" width="8.83203125" style="55"/>
-    <col min="10" max="10" width="7.33203125" style="55" customWidth="1"/>
-    <col min="11" max="11" width="8.83203125" style="55"/>
-    <col min="12" max="12" width="24.6640625" style="55" customWidth="1"/>
-    <col min="13" max="13" width="8.83203125" style="55"/>
-    <col min="14" max="14" width="10" style="60" customWidth="1"/>
-    <col min="15" max="16384" width="8.83203125" style="55"/>
+    <col min="1" max="1" width="10.83203125" style="58" customWidth="1"/>
+    <col min="2" max="2" width="12.5" style="55" customWidth="1"/>
+    <col min="3" max="3" width="7.6640625" style="53" customWidth="1"/>
+    <col min="4" max="4" width="27.33203125" style="53" customWidth="1"/>
+    <col min="5" max="5" width="22.5" style="53" customWidth="1"/>
+    <col min="6" max="6" width="7.1640625" style="56" customWidth="1"/>
+    <col min="7" max="7" width="9" style="56" customWidth="1"/>
+    <col min="8" max="8" width="7.33203125" style="56" customWidth="1"/>
+    <col min="9" max="9" width="8.83203125" style="53"/>
+    <col min="10" max="10" width="7.33203125" style="53" customWidth="1"/>
+    <col min="11" max="11" width="8.83203125" style="53"/>
+    <col min="12" max="12" width="24.6640625" style="53" customWidth="1"/>
+    <col min="13" max="13" width="8.83203125" style="53"/>
+    <col min="14" max="14" width="10" style="58" customWidth="1"/>
+    <col min="15" max="16384" width="8.83203125" style="53"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="51" t="s">
+      <c r="B1" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="52" t="s">
+      <c r="C1" s="50" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="52" t="s">
+      <c r="D1" s="50" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="52" t="s">
+      <c r="E1" s="50" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="53" t="s">
+      <c r="F1" s="51" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="53" t="s">
+      <c r="G1" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="51" t="s">
+      <c r="H1" s="49" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="52" t="s">
+      <c r="I1" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="52" t="s">
+      <c r="J1" s="50" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="52" t="s">
+      <c r="K1" s="50" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="52" t="s">
+      <c r="L1" s="50" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="52" t="s">
+      <c r="M1" s="50" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="50" t="s">
+      <c r="N1" s="48" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="54" t="s">
+      <c r="O1" s="52" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="54" t="s">
+      <c r="P1" s="52" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="54" t="s">
+      <c r="Q1" s="52" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="54" t="s">
+      <c r="R1" s="52" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="54" t="s">
+      <c r="S1" s="52" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="54" t="s">
+      <c r="T1" s="52" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="54" t="s">
+      <c r="U1" s="52" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:21" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="56"/>
-      <c r="B2" s="57" t="s">
+      <c r="A2" s="54"/>
+      <c r="B2" s="55" t="s">
         <v>5197</v>
       </c>
-      <c r="C2" s="55" t="s">
+      <c r="C2" s="53" t="s">
         <v>1100</v>
       </c>
-      <c r="D2" s="55" t="s">
+      <c r="D2" s="53" t="s">
         <v>1101</v>
       </c>
-      <c r="E2" s="55" t="s">
+      <c r="E2" s="53" t="s">
         <v>4638</v>
       </c>
-      <c r="F2" s="58">
+      <c r="F2" s="56">
         <v>1975</v>
       </c>
-      <c r="G2" s="59"/>
+      <c r="G2" s="57"/>
     </row>
     <row r="3" spans="1:21" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="56"/>
-      <c r="B3" s="57" t="s">
+      <c r="A3" s="54"/>
+      <c r="B3" s="55" t="s">
         <v>5197</v>
       </c>
-      <c r="C3" s="55" t="s">
+      <c r="C3" s="53" t="s">
         <v>1112</v>
       </c>
-      <c r="D3" s="55" t="s">
+      <c r="D3" s="53" t="s">
         <v>1113</v>
       </c>
-      <c r="E3" s="55" t="s">
+      <c r="E3" s="53" t="s">
         <v>4639</v>
       </c>
-      <c r="F3" s="58">
+      <c r="F3" s="56">
         <v>1982</v>
       </c>
-      <c r="G3" s="59"/>
+      <c r="G3" s="57"/>
     </row>
     <row r="4" spans="1:21" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A4" s="56"/>
-      <c r="B4" s="57" t="s">
+      <c r="A4" s="54"/>
+      <c r="B4" s="55" t="s">
         <v>5197</v>
       </c>
-      <c r="C4" s="55" t="s">
+      <c r="C4" s="53" t="s">
         <v>1119</v>
       </c>
-      <c r="D4" s="55" t="s">
+      <c r="D4" s="53" t="s">
         <v>1120</v>
       </c>
-      <c r="E4" s="55" t="s">
+      <c r="E4" s="53" t="s">
         <v>4640</v>
       </c>
-      <c r="F4" s="58">
+      <c r="F4" s="56">
         <v>1984</v>
       </c>
-      <c r="G4" s="59"/>
-      <c r="K4" s="61"/>
+      <c r="G4" s="57"/>
+      <c r="K4" s="59"/>
     </row>
     <row r="5" spans="1:21" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="29"/>
-      <c r="B5" s="57" t="s">
+      <c r="B5" s="55" t="s">
         <v>5199</v>
       </c>
-      <c r="C5" s="55" t="s">
+      <c r="C5" s="53" t="s">
         <v>4641</v>
       </c>
-      <c r="D5" s="55" t="s">
+      <c r="D5" s="53" t="s">
         <v>4642</v>
       </c>
-      <c r="E5" s="55" t="s">
+      <c r="E5" s="53" t="s">
         <v>4643</v>
       </c>
-      <c r="F5" s="58">
+      <c r="F5" s="56">
         <v>1958</v>
       </c>
     </row>
     <row r="6" spans="1:21" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="29"/>
-      <c r="B6" s="57" t="s">
+      <c r="B6" s="55" t="s">
         <v>5199</v>
       </c>
-      <c r="C6" s="55" t="s">
+      <c r="C6" s="53" t="s">
         <v>4645</v>
       </c>
-      <c r="D6" s="55" t="s">
+      <c r="D6" s="53" t="s">
         <v>4646</v>
       </c>
-      <c r="E6" s="55" t="s">
+      <c r="E6" s="53" t="s">
         <v>4647</v>
       </c>
-      <c r="F6" s="58">
+      <c r="F6" s="56">
         <v>1959</v>
       </c>
     </row>
     <row r="7" spans="1:21" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="29"/>
-      <c r="B7" s="57" t="s">
+      <c r="B7" s="55" t="s">
         <v>5205</v>
       </c>
-      <c r="C7" s="55" t="s">
+      <c r="C7" s="53" t="s">
         <v>4648</v>
       </c>
-      <c r="D7" s="55" t="s">
+      <c r="D7" s="53" t="s">
         <v>4649</v>
       </c>
-      <c r="E7" s="55" t="s">
+      <c r="E7" s="53" t="s">
         <v>4650</v>
       </c>
-      <c r="F7" s="58">
+      <c r="F7" s="56">
         <v>1963</v>
       </c>
     </row>
     <row r="8" spans="1:21" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="29"/>
-      <c r="B8" s="57" t="s">
+      <c r="B8" s="55" t="s">
         <v>5205</v>
       </c>
-      <c r="C8" s="55" t="s">
+      <c r="C8" s="53" t="s">
         <v>4651</v>
       </c>
-      <c r="D8" s="55" t="s">
+      <c r="D8" s="53" t="s">
         <v>4652</v>
       </c>
-      <c r="E8" s="55" t="s">
+      <c r="E8" s="53" t="s">
         <v>4653</v>
       </c>
-      <c r="F8" s="58">
+      <c r="F8" s="56">
         <v>1977</v>
       </c>
     </row>
     <row r="9" spans="1:21" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="29"/>
-      <c r="B9" s="57" t="s">
+      <c r="B9" s="55" t="s">
         <v>5201</v>
       </c>
-      <c r="C9" s="55" t="s">
+      <c r="C9" s="53" t="s">
         <v>4654</v>
       </c>
-      <c r="D9" s="55" t="s">
+      <c r="D9" s="53" t="s">
         <v>4655</v>
       </c>
-      <c r="E9" s="55" t="s">
+      <c r="E9" s="53" t="s">
         <v>4656</v>
       </c>
-      <c r="F9" s="58">
+      <c r="F9" s="56">
         <v>1953</v>
       </c>
     </row>
     <row r="10" spans="1:21" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="29"/>
-      <c r="B10" s="57" t="s">
+      <c r="B10" s="55" t="s">
         <v>5201</v>
       </c>
-      <c r="C10" s="55" t="s">
+      <c r="C10" s="53" t="s">
         <v>4658</v>
       </c>
-      <c r="D10" s="55" t="s">
+      <c r="D10" s="53" t="s">
         <v>4659</v>
       </c>
-      <c r="E10" s="55" t="s">
+      <c r="E10" s="53" t="s">
         <v>4660</v>
       </c>
-      <c r="F10" s="58">
+      <c r="F10" s="56">
         <v>1954</v>
       </c>
     </row>
     <row r="11" spans="1:21" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="29"/>
-      <c r="B11" s="57" t="s">
+      <c r="B11" s="55" t="s">
         <v>5201</v>
       </c>
-      <c r="C11" s="55" t="s">
+      <c r="C11" s="53" t="s">
         <v>4661</v>
       </c>
-      <c r="D11" s="55" t="s">
+      <c r="D11" s="53" t="s">
         <v>4662</v>
       </c>
-      <c r="E11" s="55" t="s">
+      <c r="E11" s="53" t="s">
         <v>4663</v>
       </c>
-      <c r="F11" s="58">
+      <c r="F11" s="56">
         <v>1955</v>
       </c>
     </row>
     <row r="12" spans="1:21" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="29"/>
-      <c r="B12" s="57" t="s">
+      <c r="B12" s="55" t="s">
         <v>5202</v>
       </c>
-      <c r="D12" s="55" t="s">
+      <c r="D12" s="53" t="s">
         <v>4664</v>
       </c>
-      <c r="E12" s="55" t="s">
+      <c r="E12" s="53" t="s">
         <v>4665</v>
       </c>
-      <c r="F12" s="58">
+      <c r="F12" s="56">
         <v>1960</v>
       </c>
     </row>
     <row r="13" spans="1:21" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="29"/>
-      <c r="B13" s="57" t="s">
+      <c r="B13" s="55" t="s">
         <v>5198</v>
       </c>
-      <c r="D13" s="55" t="s">
+      <c r="D13" s="53" t="s">
         <v>4666</v>
       </c>
-      <c r="E13" s="55" t="s">
+      <c r="E13" s="53" t="s">
         <v>4667</v>
       </c>
-      <c r="F13" s="58">
+      <c r="F13" s="56">
         <v>1968</v>
       </c>
     </row>
     <row r="14" spans="1:21" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="29"/>
-      <c r="B14" s="57" t="s">
+      <c r="B14" s="55" t="s">
         <v>5203</v>
       </c>
-      <c r="D14" s="55" t="s">
+      <c r="D14" s="53" t="s">
         <v>4668</v>
       </c>
-      <c r="E14" s="55" t="s">
+      <c r="E14" s="53" t="s">
         <v>4669</v>
       </c>
-      <c r="F14" s="58">
+      <c r="F14" s="56">
         <v>2013</v>
       </c>
     </row>
     <row r="15" spans="1:21" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="29"/>
-      <c r="B15" s="57" t="s">
+      <c r="B15" s="55" t="s">
         <v>5198</v>
       </c>
-      <c r="D15" s="55" t="s">
+      <c r="D15" s="53" t="s">
         <v>4670</v>
       </c>
-      <c r="E15" s="55" t="s">
+      <c r="E15" s="53" t="s">
         <v>4671</v>
       </c>
-      <c r="F15" s="58">
+      <c r="F15" s="56">
         <v>1956</v>
       </c>
     </row>
     <row r="16" spans="1:21" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="29"/>
-      <c r="B16" s="57" t="s">
+      <c r="B16" s="55" t="s">
         <v>5198</v>
       </c>
-      <c r="D16" s="55" t="s">
+      <c r="D16" s="53" t="s">
         <v>4673</v>
       </c>
-      <c r="E16" s="55" t="s">
+      <c r="E16" s="53" t="s">
         <v>4674</v>
       </c>
-      <c r="F16" s="58">
+      <c r="F16" s="56">
         <v>1966</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="29"/>
-      <c r="B17" s="57" t="s">
+      <c r="B17" s="55" t="s">
         <v>5202</v>
       </c>
-      <c r="D17" s="55" t="s">
+      <c r="D17" s="53" t="s">
         <v>4675</v>
       </c>
-      <c r="E17" s="55" t="s">
+      <c r="E17" s="53" t="s">
         <v>4676</v>
       </c>
-      <c r="F17" s="58">
+      <c r="F17" s="56">
         <v>1962</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="29"/>
-      <c r="B18" s="57" t="s">
+      <c r="B18" s="55" t="s">
         <v>5206</v>
       </c>
-      <c r="D18" s="55" t="s">
+      <c r="D18" s="53" t="s">
         <v>4677</v>
       </c>
-      <c r="E18" s="55" t="s">
+      <c r="E18" s="53" t="s">
         <v>4678</v>
       </c>
-      <c r="F18" s="58">
+      <c r="F18" s="56">
         <v>1966</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="29"/>
-      <c r="B19" s="57" t="s">
+      <c r="B19" s="55" t="s">
         <v>5198</v>
       </c>
-      <c r="D19" s="55" t="s">
+      <c r="D19" s="53" t="s">
         <v>4679</v>
       </c>
-      <c r="E19" s="55" t="s">
+      <c r="E19" s="53" t="s">
         <v>4680</v>
       </c>
-      <c r="F19" s="58">
+      <c r="F19" s="56">
         <v>1954</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="29"/>
-      <c r="B20" s="57" t="s">
+      <c r="B20" s="55" t="s">
         <v>5198</v>
       </c>
-      <c r="D20" s="55" t="s">
+      <c r="D20" s="53" t="s">
         <v>4681</v>
       </c>
-      <c r="E20" s="55" t="s">
+      <c r="E20" s="53" t="s">
         <v>4682</v>
       </c>
-      <c r="F20" s="58">
+      <c r="F20" s="56">
         <v>1960</v>
       </c>
     </row>
     <row r="21" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="29"/>
-      <c r="B21" s="57" t="s">
+      <c r="B21" s="55" t="s">
         <v>5202</v>
       </c>
-      <c r="D21" s="55" t="s">
+      <c r="D21" s="53" t="s">
         <v>4683</v>
       </c>
-      <c r="E21" s="55" t="s">
+      <c r="E21" s="53" t="s">
         <v>4684</v>
       </c>
-      <c r="F21" s="58">
+      <c r="F21" s="56">
         <v>1961</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="29"/>
-      <c r="B22" s="57" t="s">
+      <c r="B22" s="55" t="s">
         <v>5204</v>
       </c>
-      <c r="D22" s="55" t="s">
+      <c r="D22" s="53" t="s">
         <v>4685</v>
       </c>
-      <c r="E22" s="55" t="s">
+      <c r="E22" s="53" t="s">
         <v>4686</v>
       </c>
-      <c r="F22" s="58">
+      <c r="F22" s="56">
         <v>1965</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="29"/>
-      <c r="B23" s="57" t="s">
+      <c r="B23" s="55" t="s">
         <v>5202</v>
       </c>
-      <c r="D23" s="55" t="s">
+      <c r="D23" s="53" t="s">
         <v>4687</v>
       </c>
-      <c r="E23" s="55" t="s">
+      <c r="E23" s="53" t="s">
         <v>4688</v>
       </c>
-      <c r="F23" s="58">
+      <c r="F23" s="56">
         <v>1960</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="29"/>
-      <c r="B24" s="57" t="s">
+      <c r="B24" s="55" t="s">
         <v>5202</v>
       </c>
-      <c r="D24" s="55" t="s">
+      <c r="D24" s="53" t="s">
         <v>4689</v>
       </c>
-      <c r="E24" s="55" t="s">
+      <c r="E24" s="53" t="s">
         <v>4689</v>
       </c>
-      <c r="F24" s="58">
+      <c r="F24" s="56">
         <v>1968</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="29"/>
-      <c r="B25" s="57" t="s">
+      <c r="B25" s="55" t="s">
         <v>5198</v>
       </c>
-      <c r="D25" s="55" t="s">
+      <c r="D25" s="53" t="s">
         <v>4690</v>
       </c>
-      <c r="E25" s="55" t="s">
+      <c r="E25" s="53" t="s">
         <v>4691</v>
       </c>
-      <c r="F25" s="58">
+      <c r="F25" s="56">
         <v>1960</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="29"/>
-      <c r="B26" s="57" t="s">
+      <c r="B26" s="55" t="s">
         <v>5202</v>
       </c>
-      <c r="D26" s="55" t="s">
+      <c r="D26" s="53" t="s">
         <v>4692</v>
       </c>
-      <c r="E26" s="55" t="s">
+      <c r="E26" s="53" t="s">
         <v>4692</v>
       </c>
-      <c r="F26" s="58">
+      <c r="F26" s="56">
         <v>1962</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="29"/>
-      <c r="B27" s="57" t="s">
+      <c r="B27" s="55" t="s">
         <v>5198</v>
       </c>
-      <c r="D27" s="55" t="s">
+      <c r="D27" s="53" t="s">
         <v>4693</v>
       </c>
-      <c r="E27" s="55" t="s">
+      <c r="E27" s="53" t="s">
         <v>4694</v>
       </c>
-      <c r="F27" s="58">
+      <c r="F27" s="56">
         <v>1971</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="29"/>
-      <c r="B28" s="57" t="s">
+      <c r="B28" s="55" t="s">
         <v>5204</v>
       </c>
-      <c r="D28" s="55" t="s">
+      <c r="D28" s="53" t="s">
         <v>4695</v>
       </c>
-      <c r="E28" s="55" t="s">
+      <c r="E28" s="53" t="s">
         <v>4696</v>
       </c>
-      <c r="F28" s="58">
+      <c r="F28" s="56">
         <v>1971</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="29"/>
-      <c r="B29" s="57" t="s">
+      <c r="B29" s="55" t="s">
         <v>5202</v>
       </c>
-      <c r="D29" s="55" t="s">
+      <c r="D29" s="53" t="s">
         <v>4697</v>
       </c>
-      <c r="E29" s="55" t="s">
+      <c r="E29" s="53" t="s">
         <v>4698</v>
       </c>
-      <c r="F29" s="58">
+      <c r="F29" s="56">
         <v>1974</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="29"/>
-      <c r="B30" s="57" t="s">
+      <c r="B30" s="55" t="s">
         <v>5202</v>
       </c>
-      <c r="D30" s="55" t="s">
+      <c r="D30" s="53" t="s">
         <v>4699</v>
       </c>
-      <c r="E30" s="55" t="s">
+      <c r="E30" s="53" t="s">
         <v>4700</v>
       </c>
-      <c r="F30" s="58">
+      <c r="F30" s="56">
         <v>1962</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="29"/>
-      <c r="B31" s="57" t="s">
+      <c r="B31" s="55" t="s">
         <v>5202</v>
       </c>
-      <c r="D31" s="55" t="s">
+      <c r="D31" s="53" t="s">
         <v>4701</v>
       </c>
-      <c r="E31" s="55" t="s">
+      <c r="E31" s="53" t="s">
         <v>4702</v>
       </c>
-      <c r="F31" s="58">
+      <c r="F31" s="56">
         <v>1966</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="29"/>
-      <c r="B32" s="57" t="s">
+      <c r="B32" s="55" t="s">
         <v>5202</v>
       </c>
-      <c r="D32" s="55" t="s">
+      <c r="D32" s="53" t="s">
         <v>4703</v>
       </c>
-      <c r="E32" s="55" t="s">
+      <c r="E32" s="53" t="s">
         <v>4704</v>
       </c>
-      <c r="F32" s="58">
+      <c r="F32" s="56">
         <v>1998</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A33" s="29"/>
-      <c r="B33" s="57" t="s">
+      <c r="B33" s="55" t="s">
         <v>5202</v>
       </c>
-      <c r="D33" s="55" t="s">
+      <c r="D33" s="53" t="s">
         <v>4705</v>
       </c>
-      <c r="E33" s="55" t="s">
+      <c r="E33" s="53" t="s">
         <v>4706</v>
       </c>
-      <c r="F33" s="58">
+      <c r="F33" s="56">
         <v>1963</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A34" s="29"/>
-      <c r="B34" s="57" t="s">
+      <c r="B34" s="55" t="s">
         <v>5198</v>
       </c>
-      <c r="D34" s="55" t="s">
+      <c r="D34" s="53" t="s">
         <v>4707</v>
       </c>
-      <c r="E34" s="55" t="s">
+      <c r="E34" s="53" t="s">
         <v>4708</v>
       </c>
-      <c r="F34" s="58">
+      <c r="F34" s="56">
         <v>1981</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A35" s="29"/>
-      <c r="B35" s="57" t="s">
+      <c r="B35" s="55" t="s">
         <v>5202</v>
       </c>
-      <c r="D35" s="55" t="s">
+      <c r="D35" s="53" t="s">
         <v>4709</v>
       </c>
-      <c r="E35" s="55" t="s">
+      <c r="E35" s="53" t="s">
         <v>4710</v>
       </c>
-      <c r="F35" s="58">
+      <c r="F35" s="56">
         <v>1967</v>
       </c>
     </row>
     <row r="36" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A36" s="29"/>
-      <c r="B36" s="57" t="s">
+      <c r="B36" s="55" t="s">
         <v>5198</v>
       </c>
-      <c r="D36" s="55" t="s">
+      <c r="D36" s="53" t="s">
         <v>4711</v>
       </c>
-      <c r="E36" s="55" t="s">
+      <c r="E36" s="53" t="s">
         <v>4712</v>
       </c>
-      <c r="F36" s="58">
+      <c r="F36" s="56">
         <v>1959</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A37" s="29"/>
-      <c r="B37" s="57" t="s">
+      <c r="B37" s="55" t="s">
         <v>5198</v>
       </c>
-      <c r="D37" s="55" t="s">
+      <c r="D37" s="53" t="s">
         <v>4713</v>
       </c>
-      <c r="E37" s="55" t="s">
+      <c r="E37" s="53" t="s">
         <v>4714</v>
       </c>
-      <c r="F37" s="58">
+      <c r="F37" s="56">
         <v>1961</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A38" s="29"/>
-      <c r="B38" s="57" t="s">
+      <c r="B38" s="55" t="s">
         <v>5203</v>
       </c>
-      <c r="D38" s="55" t="s">
+      <c r="D38" s="53" t="s">
         <v>4715</v>
       </c>
-      <c r="E38" s="55" t="s">
+      <c r="E38" s="53" t="s">
         <v>4716</v>
       </c>
-      <c r="F38" s="58">
+      <c r="F38" s="56">
         <v>2000</v>
       </c>
     </row>
     <row r="39" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A39" s="29"/>
-      <c r="B39" s="55" t="s">
+      <c r="B39" s="53" t="s">
         <v>5200</v>
       </c>
-      <c r="D39" s="55" t="s">
+      <c r="D39" s="53" t="s">
         <v>4717</v>
       </c>
-      <c r="E39" s="55" t="s">
+      <c r="E39" s="53" t="s">
         <v>4718</v>
       </c>
-      <c r="F39" s="58">
+      <c r="F39" s="56">
         <v>1975</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A40" s="29"/>
-      <c r="B40" s="57" t="s">
+      <c r="B40" s="55" t="s">
         <v>5202</v>
       </c>
-      <c r="D40" s="55" t="s">
+      <c r="D40" s="53" t="s">
         <v>1668</v>
       </c>
-      <c r="E40" s="55" t="s">
+      <c r="E40" s="53" t="s">
         <v>4719</v>
       </c>
-      <c r="F40" s="58">
+      <c r="F40" s="56">
         <v>1974</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A41" s="29"/>
-      <c r="B41" s="57" t="s">
+      <c r="B41" s="55" t="s">
         <v>5198</v>
       </c>
-      <c r="D41" s="55" t="s">
+      <c r="D41" s="53" t="s">
         <v>4720</v>
       </c>
-      <c r="E41" s="55" t="s">
+      <c r="E41" s="53" t="s">
         <v>4721</v>
       </c>
-      <c r="F41" s="58">
+      <c r="F41" s="56">
         <v>1974</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A42" s="29"/>
-      <c r="B42" s="57" t="s">
+      <c r="B42" s="55" t="s">
         <v>5202</v>
       </c>
-      <c r="D42" s="55" t="s">
+      <c r="D42" s="53" t="s">
         <v>4722</v>
       </c>
-      <c r="E42" s="55" t="s">
+      <c r="E42" s="53" t="s">
         <v>4723</v>
       </c>
-      <c r="F42" s="58">
+      <c r="F42" s="56">
         <v>1964</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A43" s="29"/>
-      <c r="B43" s="57" t="s">
+      <c r="B43" s="55" t="s">
         <v>5198</v>
       </c>
-      <c r="D43" s="55" t="s">
+      <c r="D43" s="53" t="s">
         <v>4724</v>
       </c>
-      <c r="E43" s="55" t="s">
+      <c r="E43" s="53" t="s">
         <v>4725</v>
       </c>
-      <c r="F43" s="58">
+      <c r="F43" s="56">
         <v>1961</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A44" s="29"/>
-      <c r="B44" s="57" t="s">
+      <c r="B44" s="55" t="s">
         <v>5198</v>
       </c>
-      <c r="D44" s="55" t="s">
+      <c r="D44" s="53" t="s">
         <v>4726</v>
       </c>
-      <c r="E44" s="55" t="s">
+      <c r="E44" s="53" t="s">
         <v>4727</v>
       </c>
-      <c r="F44" s="58">
+      <c r="F44" s="56">
         <v>1960</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A45" s="29"/>
-      <c r="B45" s="57" t="s">
+      <c r="B45" s="55" t="s">
         <v>5202</v>
       </c>
-      <c r="D45" s="55" t="s">
+      <c r="D45" s="53" t="s">
         <v>4728</v>
       </c>
-      <c r="E45" s="55" t="s">
+      <c r="E45" s="53" t="s">
         <v>4729</v>
       </c>
-      <c r="F45" s="58">
+      <c r="F45" s="56">
         <v>1962</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A46" s="29"/>
-      <c r="B46" s="57" t="s">
+      <c r="B46" s="55" t="s">
         <v>5198</v>
       </c>
-      <c r="D46" s="55" t="s">
+      <c r="D46" s="53" t="s">
         <v>4730</v>
       </c>
-      <c r="E46" s="55" t="s">
+      <c r="E46" s="53" t="s">
         <v>4731</v>
       </c>
-      <c r="F46" s="58">
+      <c r="F46" s="56">
         <v>1971</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A47" s="29"/>
-      <c r="B47" s="57" t="s">
+      <c r="B47" s="55" t="s">
         <v>5198</v>
       </c>
-      <c r="D47" s="55" t="s">
+      <c r="D47" s="53" t="s">
         <v>4732</v>
       </c>
-      <c r="E47" s="55" t="s">
+      <c r="E47" s="53" t="s">
         <v>4733</v>
       </c>
-      <c r="F47" s="58">
+      <c r="F47" s="56">
         <v>1959</v>
       </c>
     </row>
     <row r="48" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A48" s="29"/>
-      <c r="B48" s="57" t="s">
+      <c r="B48" s="55" t="s">
         <v>5198</v>
       </c>
-      <c r="D48" s="55" t="s">
+      <c r="D48" s="53" t="s">
         <v>4734</v>
       </c>
-      <c r="E48" s="55" t="s">
+      <c r="E48" s="53" t="s">
         <v>4735</v>
       </c>
-      <c r="F48" s="58">
+      <c r="F48" s="56">
         <v>1958</v>
       </c>
     </row>
     <row r="49" spans="1:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A49" s="29"/>
-      <c r="B49" s="57" t="s">
+      <c r="B49" s="55" t="s">
         <v>5198</v>
       </c>
-      <c r="D49" s="55" t="s">
+      <c r="D49" s="53" t="s">
         <v>4736</v>
       </c>
-      <c r="E49" s="55" t="s">
+      <c r="E49" s="53" t="s">
         <v>4737</v>
       </c>
-      <c r="F49" s="58">
+      <c r="F49" s="56">
         <v>1960</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="D50" s="62" t="s">
+      <c r="D50" s="60" t="s">
         <v>5207</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="D51" s="62"/>
+      <c r="D51" s="60"/>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="D52" s="62"/>
+      <c r="D52" s="60"/>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="D53" s="62"/>
+      <c r="D53" s="60"/>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="D54" s="62"/>
+      <c r="D54" s="60"/>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="D55" s="62"/>
+      <c r="D55" s="60"/>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="D56" s="62"/>
+      <c r="D56" s="60"/>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="D57" s="62"/>
+      <c r="D57" s="60"/>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="D58" s="62"/>
+      <c r="D58" s="60"/>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="D59" s="62"/>
+      <c r="D59" s="60"/>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="D60" s="62"/>
+      <c r="D60" s="60"/>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="D61" s="62"/>
+      <c r="D61" s="60"/>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="D62" s="62"/>
+      <c r="D62" s="60"/>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="D63" s="62"/>
+      <c r="D63" s="60"/>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.15">
-      <c r="D64" s="62"/>
+      <c r="D64" s="60"/>
     </row>
     <row r="65" spans="4:4" x14ac:dyDescent="0.15">
-      <c r="D65" s="62"/>
+      <c r="D65" s="60"/>
     </row>
     <row r="66" spans="4:4" x14ac:dyDescent="0.15">
-      <c r="D66" s="62"/>
+      <c r="D66" s="60"/>
     </row>
     <row r="67" spans="4:4" x14ac:dyDescent="0.15">
-      <c r="D67" s="62"/>
+      <c r="D67" s="60"/>
     </row>
     <row r="68" spans="4:4" x14ac:dyDescent="0.15">
-      <c r="D68" s="62"/>
+      <c r="D68" s="60"/>
     </row>
     <row r="69" spans="4:4" x14ac:dyDescent="0.15">
-      <c r="D69" s="62"/>
+      <c r="D69" s="60"/>
     </row>
     <row r="70" spans="4:4" x14ac:dyDescent="0.15">
-      <c r="D70" s="62"/>
+      <c r="D70" s="60"/>
     </row>
     <row r="71" spans="4:4" x14ac:dyDescent="0.15">
-      <c r="D71" s="62"/>
+      <c r="D71" s="60"/>
     </row>
     <row r="72" spans="4:4" x14ac:dyDescent="0.15">
-      <c r="D72" s="62"/>
+      <c r="D72" s="60"/>
     </row>
     <row r="73" spans="4:4" x14ac:dyDescent="0.15">
-      <c r="D73" s="62"/>
+      <c r="D73" s="60"/>
     </row>
     <row r="74" spans="4:4" x14ac:dyDescent="0.15">
-      <c r="D74" s="62"/>
+      <c r="D74" s="60"/>
     </row>
     <row r="75" spans="4:4" x14ac:dyDescent="0.15">
-      <c r="D75" s="62"/>
+      <c r="D75" s="60"/>
     </row>
     <row r="76" spans="4:4" x14ac:dyDescent="0.15">
-      <c r="D76" s="62"/>
+      <c r="D76" s="60"/>
     </row>
     <row r="77" spans="4:4" x14ac:dyDescent="0.15">
-      <c r="D77" s="62"/>
+      <c r="D77" s="60"/>
     </row>
     <row r="78" spans="4:4" x14ac:dyDescent="0.15">
-      <c r="D78" s="62"/>
+      <c r="D78" s="60"/>
     </row>
     <row r="79" spans="4:4" x14ac:dyDescent="0.15">
-      <c r="D79" s="62"/>
+      <c r="D79" s="60"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:U1" xr:uid="{00000000-0009-0000-0000-00000B000000}">
@@ -32505,7 +32499,7 @@
       <c r="A43" s="14" t="s">
         <v>980</v>
       </c>
-      <c r="B43" s="46"/>
+      <c r="B43" s="45"/>
       <c r="D43" t="s">
         <v>981</v>
       </c>
@@ -35847,7 +35841,7 @@
       <c r="A44" s="14" t="s">
         <v>1373</v>
       </c>
-      <c r="B44" s="49"/>
+      <c r="B44" s="47"/>
       <c r="D44" t="s">
         <v>1374</v>
       </c>
@@ -39688,9 +39682,6 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <sheetPr>
-    <tabColor rgb="FFFF0000"/>
-  </sheetPr>
   <dimension ref="A1:V73"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
@@ -41193,7 +41184,7 @@
       <c r="A26" s="14" t="s">
         <v>2246</v>
       </c>
-      <c r="B26" s="47" t="s">
+      <c r="B26" s="46" t="s">
         <v>5178</v>
       </c>
       <c r="C26" s="37"/>
@@ -41253,7 +41244,7 @@
       <c r="A27" s="14" t="s">
         <v>2289</v>
       </c>
-      <c r="B27" s="47" t="s">
+      <c r="B27" s="46" t="s">
         <v>5178</v>
       </c>
       <c r="C27" s="37"/>
@@ -43584,10 +43575,10 @@
       <c r="K68" s="37" t="s">
         <v>28</v>
       </c>
-      <c r="L68" s="48" t="s">
+      <c r="L68" s="37" t="s">
         <v>5196</v>
       </c>
-      <c r="M68" s="48" t="s">
+      <c r="M68" s="37" t="s">
         <v>30</v>
       </c>
       <c r="N68" s="38" t="s">
@@ -45844,9 +45835,6 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <sheetPr>
-    <tabColor rgb="FFFF0000"/>
-  </sheetPr>
   <dimension ref="A1:U54"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
@@ -48699,7 +48687,7 @@
       <c r="A48" s="14" t="s">
         <v>3050</v>
       </c>
-      <c r="B48" s="22" t="s">
+      <c r="B48" s="61" t="s">
         <v>5170</v>
       </c>
       <c r="D48" t="s">
@@ -49000,7 +48988,7 @@
       <c r="G53" s="13">
         <v>8.5416666666666669E-2</v>
       </c>
-      <c r="H53" s="45">
+      <c r="H53" s="62">
         <v>7.8</v>
       </c>
       <c r="I53" t="s">

</xml_diff>